<commit_message>
Mise à jour IG 1e8281302f5014123b27b19308d074213a63f7aa
</commit_message>
<xml_diff>
--- a/structureIG/ig/StructureDefinition-fr-lm-patient-summary-document.xlsx
+++ b/structureIG/ig/StructureDefinition-fr-lm-patient-summary-document.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-22T08:07:02+00:00</t>
+    <t>2026-09-22T09:47:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -617,7 +617,7 @@
 </t>
   </si>
   <si>
-    <t>Section Points de Vigilances non codé</t>
+    <t>Section Points de Vigilances</t>
   </si>
   <si>
     <t>fr-lm-patient-summary-document.functionalStatus</t>

</xml_diff>